<commit_message>
Closing v3.0, making major architectural changes
</commit_message>
<xml_diff>
--- a/Research_Daily_Plan_v3.xlsx
+++ b/Research_Daily_Plan_v3.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rahul\Nyaymalaw 3.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C2476E6-A531-4DAD-9854-97EA5023BAE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9FED4A5-491C-4233-9C06-A8A43BF4BE4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,15 +29,12 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="172">
   <si>
     <t>Date</t>
   </si>
@@ -92,6 +89,9 @@
   </si>
   <si>
     <t>Pilot run — 10 queries through full pipeline</t>
+  </si>
+  <si>
+    <t>Not Started</t>
   </si>
   <si>
     <t>Run fast ablation modes + first threshold sweep</t>
@@ -125,9 +125,6 @@
 6. Check safety report: cat eval/results/safety/safety_report_*.json | python -m json.tool | head -20
 7. Create eval/data/system_versions.txt with all version info you collected on Day 1
 8. RECORD in a notebook: per-query time, threshold finding, ablation comparison numbers</t>
-  </si>
-  <si>
-    <t>In Progress</t>
   </si>
   <si>
     <t>Queries</t>
@@ -160,9 +157,6 @@
   · SIGALRM crash is FIXED — batch_runner uses ThreadPoolExecutor
   · Use Windows Terminal tabs instead of tmux
 </t>
-  </si>
-  <si>
-    <t>Not Started</t>
   </si>
   <si>
     <t>Run criminal domain queries (10 queries)</t>
@@ -1171,19 +1165,22 @@
     <t>Week 10 complete</t>
   </si>
   <si>
-    <t>VRAM usage:6812MiB /   8188MiB</t>
-  </si>
-  <si>
     <t>1. Open tmux: tmux new -s eval
 2. Start Ollama if not running: ollama serve &amp;
 3. Run pilot batch (takes ~30-40 min on RTX 4060):
-   python -m eval.batch_runner --queries eval/data/queries_v2.json --out eval/results/ --mode full_pipeline; python -m eval.batch_runner --queries eval/data/queries_v2.json --out eval/results/ --mode full_pipeline --limit 15
+python -m eval.batch_runner --queries eval/data/queries_v2.json --out eval/results/ --mode full_pipeline --limit 10
 4. While GPU runs, open another terminal and monitor:
    watch -n 2 nvidia-smi
 5. Note: (a) VRAM usage, (b) per-query time from log output, (c) any errors
 6. When done, check results file exists:
    ls -la eval/results/batch_full_pipeline_*.json
-7. Quick inspect: python -c "import json; d=json.load(open('eval/results/batch_full_pipeline_*.json'.replace('*','$(ls eval/results/batch_full_pipeline_*.json | head -1 | xargs basename)'))); print(f'{len(d)} results, first query took {d[0].get(\"elapsed_seconds\",0):.1f}s')"
+7. Quick inspect: python -c "import json, sys; 
+from pathlib import Path; 
+p = Path(sys.argv[1]); 
+with p.open(encoding='utf-8') as f: 
+    d = json.load(f); 
+print('{} results, first query took {:.1f}s'.format(len(d), d[0].get('elapsed_seconds', 0)))" `
+  (Get-ChildItem eval\results\batch_full_pipeline_*.json | Sort-Object LastWriteTime -Descending | Select-Object -First 1 -ExpandProperty FullName)
 NOTE (Windows 11 fix): batch_runner.py SIGALRM crash has been resolved. Uses concurrent.futures.ThreadPoolExecutor — no SIGALRM errors expected on Windows.</t>
   </si>
 </sst>
@@ -1425,7 +1422,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1515,8 +1512,9 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1805,14 +1803,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="31"/>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
+      <c r="A1" s="33"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
     </row>
     <row r="2" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="32"/>
+      <c r="A2" s="31"/>
       <c r="B2" s="32"/>
       <c r="C2" s="32"/>
       <c r="D2" s="32"/>
@@ -1838,7 +1836,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>46072</v>
       </c>
@@ -1848,7 +1846,7 @@
       <c r="C5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="12" t="s">
         <v>8</v>
       </c>
       <c r="E5" s="7" t="s">
@@ -1870,14 +1868,12 @@
         <v>11</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>172</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F6" s="12"/>
     </row>
     <row r="7" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
@@ -1888,13 +1884,13 @@
         <v>6</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F7" s="12"/>
     </row>
@@ -1907,13 +1903,13 @@
         <v>6</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F8" s="12"/>
     </row>
@@ -1932,7 +1928,7 @@
         <v>19</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F9" s="12"/>
     </row>
@@ -1945,13 +1941,13 @@
         <v>17</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="6" t="s">
-        <v>22</v>
-      </c>
       <c r="E10" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F10" s="12"/>
     </row>
@@ -1964,13 +1960,13 @@
         <v>17</v>
       </c>
       <c r="C11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="12" t="s">
-        <v>24</v>
-      </c>
       <c r="E11" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F11" s="12"/>
     </row>
@@ -1983,13 +1979,13 @@
         <v>17</v>
       </c>
       <c r="C12" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>26</v>
-      </c>
       <c r="E12" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F12" s="12"/>
     </row>
@@ -2002,13 +1998,13 @@
         <v>17</v>
       </c>
       <c r="C13" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="6" t="s">
-        <v>28</v>
-      </c>
       <c r="E13" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F13" s="12"/>
     </row>
@@ -2021,13 +2017,13 @@
         <v>17</v>
       </c>
       <c r="C14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="6" t="s">
-        <v>30</v>
-      </c>
       <c r="E14" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F14" s="12"/>
     </row>
@@ -2040,13 +2036,13 @@
         <v>17</v>
       </c>
       <c r="C15" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>32</v>
-      </c>
       <c r="E15" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F15" s="12"/>
     </row>
@@ -2059,13 +2055,13 @@
         <v>17</v>
       </c>
       <c r="C16" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D16" s="6" t="s">
-        <v>34</v>
-      </c>
       <c r="E16" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F16" s="12"/>
     </row>
@@ -2078,13 +2074,13 @@
         <v>17</v>
       </c>
       <c r="C17" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>36</v>
-      </c>
       <c r="E17" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F17" s="12"/>
     </row>
@@ -2094,16 +2090,16 @@
         <v>46085</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="6" t="s">
-        <v>39</v>
-      </c>
       <c r="E18" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F18" s="12"/>
     </row>
@@ -2116,13 +2112,13 @@
         <v>17</v>
       </c>
       <c r="C19" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="D19" s="6" t="s">
-        <v>41</v>
-      </c>
       <c r="E19" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F19" s="12"/>
     </row>
@@ -2135,13 +2131,13 @@
         <v>17</v>
       </c>
       <c r="C20" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="D20" s="6" t="s">
-        <v>43</v>
-      </c>
       <c r="E20" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F20" s="12"/>
     </row>
@@ -2154,13 +2150,13 @@
         <v>17</v>
       </c>
       <c r="C21" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D21" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="D21" s="6" t="s">
-        <v>45</v>
-      </c>
       <c r="E21" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F21" s="12"/>
     </row>
@@ -2170,16 +2166,16 @@
         <v>46089</v>
       </c>
       <c r="B22" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="D22" s="6" t="s">
-        <v>48</v>
-      </c>
       <c r="E22" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F22" s="12"/>
     </row>
@@ -2189,16 +2185,16 @@
         <v>46090</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C23" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D23" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D23" s="6" t="s">
-        <v>50</v>
-      </c>
       <c r="E23" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F23" s="12"/>
     </row>
@@ -2208,16 +2204,16 @@
         <v>46091</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C24" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D24" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D24" s="6" t="s">
-        <v>52</v>
-      </c>
       <c r="E24" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F24" s="12"/>
     </row>
@@ -2227,16 +2223,16 @@
         <v>46092</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C25" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="D25" s="6" t="s">
-        <v>54</v>
-      </c>
       <c r="E25" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F25" s="12"/>
     </row>
@@ -2246,16 +2242,16 @@
         <v>46093</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C26" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="6" t="s">
-        <v>56</v>
-      </c>
       <c r="E26" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F26" s="12"/>
     </row>
@@ -2265,16 +2261,16 @@
         <v>46094</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C27" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D27" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D27" s="6" t="s">
-        <v>58</v>
-      </c>
       <c r="E27" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F27" s="12"/>
     </row>
@@ -2284,16 +2280,16 @@
         <v>46095</v>
       </c>
       <c r="B28" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="D28" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="D28" s="6" t="s">
-        <v>61</v>
-      </c>
       <c r="E28" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F28" s="12"/>
     </row>
@@ -2303,16 +2299,16 @@
         <v>46096</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C29" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D29" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D29" s="6" t="s">
-        <v>63</v>
-      </c>
       <c r="E29" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F29" s="12"/>
     </row>
@@ -2322,16 +2318,16 @@
         <v>46097</v>
       </c>
       <c r="B30" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C30" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="D30" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D30" s="6" t="s">
-        <v>66</v>
-      </c>
       <c r="E30" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F30" s="12"/>
     </row>
@@ -2341,16 +2337,16 @@
         <v>46098</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C31" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D31" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="D31" s="6" t="s">
-        <v>68</v>
-      </c>
       <c r="E31" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F31" s="12"/>
     </row>
@@ -2360,16 +2356,16 @@
         <v>46099</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C32" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D32" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="D32" s="6" t="s">
-        <v>70</v>
-      </c>
       <c r="E32" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F32" s="12"/>
     </row>
@@ -2379,16 +2375,16 @@
         <v>46100</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C33" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D33" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="D33" s="6" t="s">
-        <v>72</v>
-      </c>
       <c r="E33" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F33" s="12"/>
     </row>
@@ -2398,16 +2394,16 @@
         <v>46101</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C34" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D34" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="D34" s="6" t="s">
-        <v>74</v>
-      </c>
       <c r="E34" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F34" s="12"/>
     </row>
@@ -2417,16 +2413,16 @@
         <v>46102</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C35" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D35" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="D35" s="6" t="s">
-        <v>76</v>
-      </c>
       <c r="E35" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F35" s="12"/>
     </row>
@@ -2436,16 +2432,16 @@
         <v>46103</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C36" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D36" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="D36" s="6" t="s">
-        <v>78</v>
-      </c>
       <c r="E36" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F36" s="12"/>
     </row>
@@ -2455,16 +2451,16 @@
         <v>46104</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C37" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D37" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D37" s="6" t="s">
-        <v>80</v>
-      </c>
       <c r="E37" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F37" s="12"/>
     </row>
@@ -2474,16 +2470,16 @@
         <v>46105</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C38" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D38" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="D38" s="6" t="s">
-        <v>82</v>
-      </c>
       <c r="E38" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F38" s="12"/>
     </row>
@@ -2493,16 +2489,16 @@
         <v>46106</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C39" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D39" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="D39" s="6" t="s">
-        <v>84</v>
-      </c>
       <c r="E39" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F39" s="12"/>
     </row>
@@ -2512,16 +2508,16 @@
         <v>46107</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C40" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D40" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="D40" s="6" t="s">
-        <v>86</v>
-      </c>
       <c r="E40" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F40" s="12"/>
     </row>
@@ -2531,16 +2527,16 @@
         <v>46108</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C41" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D41" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="D41" s="6" t="s">
-        <v>88</v>
-      </c>
       <c r="E41" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F41" s="12"/>
     </row>
@@ -2550,16 +2546,16 @@
         <v>46109</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C42" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D42" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="D42" s="6" t="s">
-        <v>90</v>
-      </c>
       <c r="E42" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F42" s="12"/>
     </row>
@@ -2569,16 +2565,16 @@
         <v>46110</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C43" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D43" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="D43" s="6" t="s">
-        <v>92</v>
-      </c>
       <c r="E43" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F43" s="12"/>
     </row>
@@ -2588,16 +2584,16 @@
         <v>46111</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C44" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D44" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="D44" s="6" t="s">
-        <v>94</v>
-      </c>
       <c r="E44" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F44" s="12"/>
     </row>
@@ -2607,16 +2603,16 @@
         <v>46112</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C45" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D45" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="D45" s="6" t="s">
-        <v>96</v>
-      </c>
       <c r="E45" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F45" s="12"/>
     </row>
@@ -2626,16 +2622,16 @@
         <v>46113</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C46" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D46" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="D46" s="6" t="s">
-        <v>98</v>
-      </c>
       <c r="E46" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F46" s="12"/>
     </row>
@@ -2645,16 +2641,16 @@
         <v>46114</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C47" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D47" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="D47" s="6" t="s">
-        <v>100</v>
-      </c>
       <c r="E47" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F47" s="12"/>
     </row>
@@ -2664,16 +2660,16 @@
         <v>46115</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C48" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D48" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="D48" s="6" t="s">
-        <v>102</v>
-      </c>
       <c r="E48" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F48" s="12"/>
     </row>
@@ -2683,16 +2679,16 @@
         <v>46116</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C49" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D49" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="D49" s="6" t="s">
-        <v>104</v>
-      </c>
       <c r="E49" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F49" s="12"/>
     </row>
@@ -2702,16 +2698,16 @@
         <v>46117</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C50" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D50" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="D50" s="6" t="s">
-        <v>106</v>
-      </c>
       <c r="E50" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F50" s="12"/>
     </row>
@@ -2721,16 +2717,16 @@
         <v>46118</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C51" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="D51" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="D51" s="6" t="s">
-        <v>108</v>
-      </c>
       <c r="E51" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F51" s="12"/>
     </row>
@@ -2740,16 +2736,16 @@
         <v>46119</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C52" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D52" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="D52" s="6" t="s">
-        <v>110</v>
-      </c>
       <c r="E52" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F52" s="12"/>
     </row>
@@ -2759,16 +2755,16 @@
         <v>46120</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C53" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="D53" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="D53" s="6" t="s">
-        <v>112</v>
-      </c>
       <c r="E53" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F53" s="12"/>
     </row>
@@ -2778,16 +2774,16 @@
         <v>46121</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C54" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="D54" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="D54" s="6" t="s">
-        <v>114</v>
-      </c>
       <c r="E54" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F54" s="12"/>
     </row>
@@ -2797,16 +2793,16 @@
         <v>46122</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C55" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D55" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="D55" s="6" t="s">
-        <v>116</v>
-      </c>
       <c r="E55" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F55" s="12"/>
     </row>
@@ -2816,16 +2812,16 @@
         <v>46123</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C56" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="D56" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="D56" s="6" t="s">
-        <v>118</v>
-      </c>
       <c r="E56" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F56" s="12"/>
     </row>
@@ -2835,16 +2831,16 @@
         <v>46124</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C57" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D57" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="D57" s="6" t="s">
-        <v>120</v>
-      </c>
       <c r="E57" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F57" s="12"/>
     </row>
@@ -2854,16 +2850,16 @@
         <v>46125</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C58" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D58" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="D58" s="6" t="s">
-        <v>122</v>
-      </c>
       <c r="E58" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F58" s="12"/>
     </row>
@@ -2873,16 +2869,16 @@
         <v>46126</v>
       </c>
       <c r="B59" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C59" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="C59" s="5" t="s">
+      <c r="D59" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="D59" s="6" t="s">
-        <v>125</v>
-      </c>
       <c r="E59" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F59" s="12"/>
     </row>
@@ -2892,16 +2888,16 @@
         <v>46127</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C60" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D60" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="D60" s="6" t="s">
-        <v>127</v>
-      </c>
       <c r="E60" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F60" s="12"/>
     </row>
@@ -2911,16 +2907,16 @@
         <v>46128</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C61" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="D61" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="D61" s="6" t="s">
-        <v>129</v>
-      </c>
       <c r="E61" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F61" s="12"/>
     </row>
@@ -2930,16 +2926,16 @@
         <v>46129</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C62" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="D62" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="D62" s="6" t="s">
-        <v>131</v>
-      </c>
       <c r="E62" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F62" s="12"/>
     </row>
@@ -2949,16 +2945,16 @@
         <v>46130</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C63" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D63" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="D63" s="6" t="s">
-        <v>133</v>
-      </c>
       <c r="E63" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F63" s="12"/>
     </row>
@@ -2968,16 +2964,16 @@
         <v>46131</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C64" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D64" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="D64" s="6" t="s">
-        <v>135</v>
-      </c>
       <c r="E64" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F64" s="12"/>
     </row>
@@ -2987,16 +2983,16 @@
         <v>46132</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C65" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="D65" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="D65" s="6" t="s">
-        <v>137</v>
-      </c>
       <c r="E65" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F65" s="12"/>
     </row>
@@ -3006,16 +3002,16 @@
         <v>46133</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C66" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D66" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="D66" s="6" t="s">
-        <v>139</v>
-      </c>
       <c r="E66" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F66" s="12"/>
     </row>
@@ -3025,16 +3021,16 @@
         <v>46134</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C67" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="D67" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="D67" s="6" t="s">
-        <v>141</v>
-      </c>
       <c r="E67" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F67" s="12"/>
     </row>
@@ -3044,16 +3040,16 @@
         <v>46135</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C68" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="D68" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="D68" s="6" t="s">
-        <v>143</v>
-      </c>
       <c r="E68" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F68" s="12"/>
     </row>
@@ -3063,28 +3059,28 @@
         <v>46136</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C69" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="D69" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="D69" s="6" t="s">
-        <v>145</v>
-      </c>
       <c r="E69" s="7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F69" s="12"/>
     </row>
     <row r="71" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C71" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="E1:E1048576 F4">
     <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
@@ -3118,34 +3114,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
-        <v>147</v>
-      </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
+      <c r="A1" s="34" t="s">
+        <v>146</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="D3" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="E3" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="F3" s="15" t="s">
         <v>151</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3153,10 +3149,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="17" t="s">
+        <v>152</v>
+      </c>
+      <c r="C4" s="18" t="s">
         <v>153</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>154</v>
       </c>
       <c r="D4" s="19">
         <v>20</v>
@@ -3165,7 +3161,7 @@
         <v>2</v>
       </c>
       <c r="F4" s="21" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3173,10 +3169,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="C5" s="18" t="s">
         <v>156</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>157</v>
       </c>
       <c r="D5" s="19">
         <v>20</v>
@@ -3185,7 +3181,7 @@
         <v>5</v>
       </c>
       <c r="F5" s="21" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3193,10 +3189,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D6" s="19">
         <v>20</v>
@@ -3205,7 +3201,7 @@
         <v>2</v>
       </c>
       <c r="F6" s="21" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3213,10 +3209,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D7" s="19">
         <v>20</v>
@@ -3225,7 +3221,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3233,10 +3229,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D8" s="19">
         <v>20</v>
@@ -3245,7 +3241,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="21" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3253,10 +3249,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D9" s="19">
         <v>20</v>
@@ -3265,7 +3261,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="21" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3273,10 +3269,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D10" s="19">
         <v>20</v>
@@ -3285,7 +3281,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="21" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3293,10 +3289,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D11" s="19">
         <v>20</v>
@@ -3305,7 +3301,7 @@
         <v>0</v>
       </c>
       <c r="F11" s="21" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3313,10 +3309,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="25" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D12" s="19">
         <v>20</v>
@@ -3325,7 +3321,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="21" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3333,10 +3329,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="25" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D13" s="19">
         <v>4</v>
@@ -3345,7 +3341,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="21" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>